<commit_message>
[NEW] Update credits, audiomixer
</commit_message>
<xml_diff>
--- a/VNFramework/Assets/StreamingAssets/story/zh/Test.xlsx
+++ b/VNFramework/Assets/StreamingAssets/story/zh/Test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="28800" windowHeight="11460"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1268,6 +1268,9 @@
       <c r="C5" t="s">
         <v>21</v>
       </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
       <c r="G5" t="s">
         <v>24</v>
       </c>
@@ -1405,6 +1408,9 @@
       </c>
       <c r="C9" t="s">
         <v>21</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>

</xml_diff>